<commit_message>
tambahkan fitur upload gambar di halaman edit tamu
</commit_message>
<xml_diff>
--- a/laporan Buku Tamu.xlsx
+++ b/laporan Buku Tamu.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>No</t>
   </si>
@@ -41,28 +41,16 @@
     <t>2026-08-28</t>
   </si>
   <si>
-    <t>fas</t>
-  </si>
-  <si>
-    <t>alafa</t>
-  </si>
-  <si>
-    <t>09q4276ry</t>
-  </si>
-  <si>
-    <t>marc</t>
-  </si>
-  <si>
-    <t>fwscsvw</t>
-  </si>
-  <si>
-    <t>sahfajbcbasfgcbas</t>
-  </si>
-  <si>
-    <t>iuasgfbsabc</t>
-  </si>
-  <si>
-    <t>dafasf</t>
+    <t>hafizh</t>
+  </si>
+  <si>
+    <t>fjasujabs</t>
+  </si>
+  <si>
+    <t>0987654321</t>
+  </si>
+  <si>
+    <t>ujsfb</t>
   </si>
   <si>
     <t>latihan</t>
@@ -71,7 +59,10 @@
     <t>Hafizh Maulana Yusufasdhasd</t>
   </si>
   <si>
-    <t>klafjssac</t>
+    <t>ugaksjfbcjasnc</t>
+  </si>
+  <si>
+    <t>main</t>
   </si>
 </sst>
 </file>
@@ -411,7 +402,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -473,37 +464,14 @@
       <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="E3">
-        <v>9999999999</v>
+      <c r="E3" t="s">
+        <v>10</v>
       </c>
       <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
         <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4">
-        <v>123456789</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pengecekan vitur dan fix_v1
</commit_message>
<xml_diff>
--- a/laporan Buku Tamu.xlsx
+++ b/laporan Buku Tamu.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
   <si>
     <t>No</t>
   </si>
@@ -38,31 +38,37 @@
     <t>KEPENTINGAN</t>
   </si>
   <si>
-    <t>2026-08-28</t>
-  </si>
-  <si>
-    <t>hafizh</t>
-  </si>
-  <si>
-    <t>fjasujabs</t>
-  </si>
-  <si>
-    <t>0987654321</t>
-  </si>
-  <si>
-    <t>ujsfb</t>
+    <t>2026-08-25</t>
+  </si>
+  <si>
+    <t>Eji Putra</t>
+  </si>
+  <si>
+    <t>Jl.karangtengah</t>
+  </si>
+  <si>
+    <t>089500100020</t>
+  </si>
+  <si>
+    <t>fikri</t>
+  </si>
+  <si>
+    <t>ngopi</t>
+  </si>
+  <si>
+    <t>Hafizh Maulana Yusuf</t>
+  </si>
+  <si>
+    <t>Jl.by pass</t>
+  </si>
+  <si>
+    <t>089502278388</t>
+  </si>
+  <si>
+    <t>marc</t>
   </si>
   <si>
     <t>latihan</t>
-  </si>
-  <si>
-    <t>Hafizh Maulana Yusufasdhasd</t>
-  </si>
-  <si>
-    <t>ugaksjfbcjasnc</t>
-  </si>
-  <si>
-    <t>main</t>
   </si>
 </sst>
 </file>
@@ -465,13 +471,13 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>